<commit_message>
Register the landscape boundaries as records (MFL-2026-098 to 105)
Eight living landscapes had their boundary only as a STAC collection asset
and in release boundaries-2026-10-14, so the catalogue showed no boundary for
them under Boundaries / admin units. Each now has a dataset record that links
to its zip in that release, with the source, licence wording and credit from
spec/boundary_provenance.json.

The eight ids join THIRD_PARTY_RIGHTS, so their STAC contact is
point-of-contact rather than licensor: the rights stay with GADM, WWF
(HydroSHEDS), the World Bank and INEI.

IND-CH, MEK-3S and TUN-NW are left out: they appear to be registered already
(000, 050, 032), pending confirmation.

102 records; STAC 115/115 valid.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -20,7 +20,7 @@
     <definedName name="MOSAIC_Access">Reference!$I$2:$I$4</definedName>
     <definedName name="MOSAIC_Migration">Reference!$O$2:$O$3</definedName>
     <definedName name="MOSAIC_UpdFreq">Reference!$Q$2:$Q$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1221,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W96"/>
+  <dimension ref="A1:W104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10744,8 +10744,880 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-098</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>N'Zi Watershed living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>CIV-NZ — N'Zi Watershed</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I97" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J97" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K97" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L97" s="8" t="inlineStr">
+        <is>
+          <t>Source terms (https://data.hydrosheds.org/file/technical-documentation/HydroSHEDS_TechDoc_v1_4.pdf)</t>
+        </is>
+      </c>
+      <c r="M97" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N97" s="8" t="inlineStr">
+        <is>
+          <t>CIV-NZ_NZi_Watershed_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O97" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P97" s="8" t="n"/>
+      <c r="Q97" s="8" t="n"/>
+      <c r="R97" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the N'Zi Watershed living landscape (CIV-NZ), used to define the landscape across the catalogue. Source: HydroBASINS v1c, level 6, basin HYBAS_ID 1060982320 (PFAF_ID 145402), unmodified. HydroSHEDS version 1, World Wildlife Fund (WWF). Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S97" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T97" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U97" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V97" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/CIV-NZ_NZi_Watershed_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W97" s="8" t="inlineStr">
+        <is>
+          <t>19 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-099</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>Cumbal (Nariño) living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
+        <is>
+          <t>COL-CUM — Cumbal (Nariño)</t>
+        </is>
+      </c>
+      <c r="F98" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G98" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H98" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I98" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J98" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K98" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L98" s="10" t="inlineStr">
+        <is>
+          <t>No licence stated by the source</t>
+        </is>
+      </c>
+      <c r="M98" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N98" s="10" t="inlineStr">
+        <is>
+          <t>COL-CUM_Cumbal_Narino_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O98" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P98" s="10" t="n"/>
+      <c r="Q98" s="10" t="n"/>
+      <c r="R98" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Cumbal (Nariño) living landscape (COL-CUM), used to define the landscape across the catalogue. Source: Nine veredas of the Cumbal indigenous reserve area (Tasmag, Quilismal, Boyera, Cuaical, Cuaspud Grande, Llano de Piedras, Cuetial, Guan, San Martin-Miraflores), layer 'Cumbal_veredas_wgs84' compiled by Javier Ochoa (CIP). Original source to be confirmed. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S98" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T98" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U98" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V98" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/COL-CUM_Cumbal_Narino_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W98" s="10" t="inlineStr">
+        <is>
+          <t>12 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-100</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Omo-Gibe Basin living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>ETH-OG — Omo-Gibe Basin</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H99" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I99" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J99" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K99" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L99" s="8" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="M99" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N99" s="8" t="inlineStr">
+        <is>
+          <t>ETH-OG_Omo-Gibe_Basin_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O99" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P99" s="8" t="n"/>
+      <c r="Q99" s="8" t="n"/>
+      <c r="R99" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Omo-Gibe Basin living landscape (ETH-OG), used to define the landscape across the catalogue. Source: Ethiopia River Basins (eth_basins), World Bank Group, World Bank Data Catalog dataset 0040202: Omo basin polygon (79,549 km2). Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S99" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T99" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U99" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V99" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/ETH-OG_Omo-Gibe_Basin_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W99" s="8" t="inlineStr">
+        <is>
+          <t>50 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-101</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>LEILA (Southern Kenya Rangelands) living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LEI — LEILA (Southern Kenya Rangelands)</t>
+        </is>
+      </c>
+      <c r="F100" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G100" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H100" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J100" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K100" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L100" s="10" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M100" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N100" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LEI_LEILA_Southern_Kenya_Rangelands_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O100" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P100" s="10" t="n"/>
+      <c r="Q100" s="10" t="n"/>
+      <c r="R100" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the LEILA (Southern Kenya Rangelands) living landscape (KEN-LEI), used to define the landscape across the catalogue. Source: GADM 4.1, level 1: counties Kajiado (KEN.10_1), Kiambu (KEN.13_1), Machakos (KEN.22_1) and Makueni (KEN.23_1), unmodified. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S100" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T100" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U100" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V100" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/KEN-LEI_LEILA_Southern_Kenya_Rangelands_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W100" s="10" t="inlineStr">
+        <is>
+          <t>315 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-102</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>Lake Victoria Basin (Kenya) living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G101" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H101" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I101" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J101" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K101" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L101" s="8" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M101" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N101" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB_Lake_Victoria_Basin_Kenya_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O101" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P101" s="8" t="n"/>
+      <c r="Q101" s="8" t="n"/>
+      <c r="R101" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Lake Victoria Basin (Kenya) living landscape (KEN-LVB), used to define the landscape across the catalogue. Source: GADM 4.1, level 1: counties Kakamega (KEN.11_1), Kisumu (KEN.17_1), Siaya (KEN.38_1) and Vihiga (KEN.45_1), unmodified. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S101" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T101" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U101" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V101" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/KEN-LVB_Lake_Victoria_Basin_Kenya_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W101" s="8" t="inlineStr">
+        <is>
+          <t>117 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-103</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>Pucallpa – Ucayali living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>PER-PCL — Pucallpa – Ucayali</t>
+        </is>
+      </c>
+      <c r="F102" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G102" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H102" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I102" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J102" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K102" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L102" s="10" t="inlineStr">
+        <is>
+          <t>No licence stated by the source</t>
+        </is>
+      </c>
+      <c r="M102" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N102" s="10" t="inlineStr">
+        <is>
+          <t>PER-PCL_Pucallpa_Ucayali_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O102" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P102" s="10" t="n"/>
+      <c r="Q102" s="10" t="n"/>
+      <c r="R102" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Pucallpa – Ucayali living landscape (PER-PCL), used to define the landscape across the catalogue. Source: INEI referential census district limits (cartography of the V Censo Nacional Economico 2022; 'Distrital' layer, ide.inei.gob.pe): 11 whole districts of Coronel Portillo and Padre Abad provinces (Ucayali) and a clipped part of Calleria. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S102" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T102" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U102" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V102" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/PER-PCL_Pucallpa_Ucayali_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W102" s="10" t="inlineStr">
+        <is>
+          <t>82 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-104</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>Fatick Department living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>SEN-FK — Fatick Department</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J103" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K103" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L103" s="8" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M103" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N103" s="8" t="inlineStr">
+        <is>
+          <t>SEN-FK_Fatick_Department_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O103" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P103" s="8" t="n"/>
+      <c r="Q103" s="8" t="n"/>
+      <c r="R103" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Fatick Department living landscape (SEN-FK), used to define the landscape across the catalogue. Source: GADM: level 2 unit Fatick departement (GADM v2 attribute schema; geometry identical to GADM 3.6 and 4.1 SEN.3.1_1). Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S103" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T103" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U103" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V103" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/SEN-FK_Fatick_Department_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W103" s="8" t="inlineStr">
+        <is>
+          <t>16 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-105</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Mbire – Lower Zambezi Valley living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>ZWE-MB — Mbire – Lower Zambezi Valley</t>
+        </is>
+      </c>
+      <c r="F104" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G104" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H104" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I104" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J104" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K104" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L104" s="10" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M104" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N104" s="10" t="inlineStr">
+        <is>
+          <t>ZWE-MB_Mbire_Lower_Zambezi_Valley_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O104" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P104" s="10" t="n"/>
+      <c r="Q104" s="10" t="n"/>
+      <c r="R104" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Mbire – Lower Zambezi Valley living landscape (ZWE-MB), used to define the landscape across the catalogue. Source: GADM 4.1, level 3: all 112 wards of the districts Mbire, Centenary/Muzarabani and Mount Darwin (Mashonaland Central) and Hurungwe (Mashonaland West), unmodified. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S104" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T104" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U104" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V104" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/ZWE-MB_Mbire_Lower_Zambezi_Valley_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W104" s="10" t="inlineStr">
+        <is>
+          <t>185 KB</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:W96"/>
+  <autoFilter ref="A2:W104"/>
   <conditionalFormatting sqref="K3:K300">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Open"</formula>

</xml_diff>

<commit_message>
Register the landscape boundaries as records (MFL-2026-098 to 105) (#3)
Eight living landscapes had their boundary only as a STAC collection asset
and in release boundaries-2026-10-14, so the catalogue showed no boundary for
them under Boundaries / admin units. Each now has a dataset record that links
to its zip in that release, with the source, licence wording and credit from
spec/boundary_provenance.json.

The eight ids join THIRD_PARTY_RIGHTS, so their STAC contact is
point-of-contact rather than licensor: the rights stay with GADM, WWF
(HydroSHEDS), the World Bank and INEI.

IND-CH, MEK-3S and TUN-NW are left out: they appear to be registered already
(000, 050, 032), pending confirmation.

102 records; STAC 115/115 valid.

Co-authored-by: lizciat <l.llanos@cgiar.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -20,7 +20,7 @@
     <definedName name="MOSAIC_Access">Reference!$I$2:$I$4</definedName>
     <definedName name="MOSAIC_Migration">Reference!$O$2:$O$3</definedName>
     <definedName name="MOSAIC_UpdFreq">Reference!$Q$2:$Q$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1221,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W96"/>
+  <dimension ref="A1:W104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10744,8 +10744,880 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-098</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>N'Zi Watershed living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>CIV-NZ — N'Zi Watershed</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I97" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J97" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K97" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L97" s="8" t="inlineStr">
+        <is>
+          <t>Source terms (https://data.hydrosheds.org/file/technical-documentation/HydroSHEDS_TechDoc_v1_4.pdf)</t>
+        </is>
+      </c>
+      <c r="M97" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N97" s="8" t="inlineStr">
+        <is>
+          <t>CIV-NZ_NZi_Watershed_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O97" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P97" s="8" t="n"/>
+      <c r="Q97" s="8" t="n"/>
+      <c r="R97" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the N'Zi Watershed living landscape (CIV-NZ), used to define the landscape across the catalogue. Source: HydroBASINS v1c, level 6, basin HYBAS_ID 1060982320 (PFAF_ID 145402), unmodified. HydroSHEDS version 1, World Wildlife Fund (WWF). Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S97" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T97" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U97" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V97" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/CIV-NZ_NZi_Watershed_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W97" s="8" t="inlineStr">
+        <is>
+          <t>19 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-099</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>Cumbal (Nariño) living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
+        <is>
+          <t>COL-CUM — Cumbal (Nariño)</t>
+        </is>
+      </c>
+      <c r="F98" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G98" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H98" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I98" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J98" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K98" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L98" s="10" t="inlineStr">
+        <is>
+          <t>No licence stated by the source</t>
+        </is>
+      </c>
+      <c r="M98" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N98" s="10" t="inlineStr">
+        <is>
+          <t>COL-CUM_Cumbal_Narino_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O98" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P98" s="10" t="n"/>
+      <c r="Q98" s="10" t="n"/>
+      <c r="R98" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Cumbal (Nariño) living landscape (COL-CUM), used to define the landscape across the catalogue. Source: Nine veredas of the Cumbal indigenous reserve area (Tasmag, Quilismal, Boyera, Cuaical, Cuaspud Grande, Llano de Piedras, Cuetial, Guan, San Martin-Miraflores), layer 'Cumbal_veredas_wgs84' compiled by Javier Ochoa (CIP). Original source to be confirmed. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S98" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T98" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U98" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V98" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/COL-CUM_Cumbal_Narino_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W98" s="10" t="inlineStr">
+        <is>
+          <t>12 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-100</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Omo-Gibe Basin living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>ETH-OG — Omo-Gibe Basin</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H99" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I99" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J99" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K99" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L99" s="8" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="M99" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N99" s="8" t="inlineStr">
+        <is>
+          <t>ETH-OG_Omo-Gibe_Basin_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O99" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P99" s="8" t="n"/>
+      <c r="Q99" s="8" t="n"/>
+      <c r="R99" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Omo-Gibe Basin living landscape (ETH-OG), used to define the landscape across the catalogue. Source: Ethiopia River Basins (eth_basins), World Bank Group, World Bank Data Catalog dataset 0040202: Omo basin polygon (79,549 km2). Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S99" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T99" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U99" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V99" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/ETH-OG_Omo-Gibe_Basin_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W99" s="8" t="inlineStr">
+        <is>
+          <t>50 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-101</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>LEILA (Southern Kenya Rangelands) living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LEI — LEILA (Southern Kenya Rangelands)</t>
+        </is>
+      </c>
+      <c r="F100" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G100" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H100" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J100" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K100" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L100" s="10" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M100" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N100" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LEI_LEILA_Southern_Kenya_Rangelands_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O100" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P100" s="10" t="n"/>
+      <c r="Q100" s="10" t="n"/>
+      <c r="R100" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the LEILA (Southern Kenya Rangelands) living landscape (KEN-LEI), used to define the landscape across the catalogue. Source: GADM 4.1, level 1: counties Kajiado (KEN.10_1), Kiambu (KEN.13_1), Machakos (KEN.22_1) and Makueni (KEN.23_1), unmodified. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S100" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T100" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U100" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V100" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/KEN-LEI_LEILA_Southern_Kenya_Rangelands_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W100" s="10" t="inlineStr">
+        <is>
+          <t>315 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-102</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>Lake Victoria Basin (Kenya) living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G101" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H101" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I101" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J101" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K101" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L101" s="8" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M101" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N101" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB_Lake_Victoria_Basin_Kenya_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O101" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P101" s="8" t="n"/>
+      <c r="Q101" s="8" t="n"/>
+      <c r="R101" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Lake Victoria Basin (Kenya) living landscape (KEN-LVB), used to define the landscape across the catalogue. Source: GADM 4.1, level 1: counties Kakamega (KEN.11_1), Kisumu (KEN.17_1), Siaya (KEN.38_1) and Vihiga (KEN.45_1), unmodified. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S101" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T101" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U101" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V101" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/KEN-LVB_Lake_Victoria_Basin_Kenya_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W101" s="8" t="inlineStr">
+        <is>
+          <t>117 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-103</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>Pucallpa – Ucayali living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>PER-PCL — Pucallpa – Ucayali</t>
+        </is>
+      </c>
+      <c r="F102" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G102" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H102" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I102" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J102" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K102" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L102" s="10" t="inlineStr">
+        <is>
+          <t>No licence stated by the source</t>
+        </is>
+      </c>
+      <c r="M102" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N102" s="10" t="inlineStr">
+        <is>
+          <t>PER-PCL_Pucallpa_Ucayali_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O102" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P102" s="10" t="n"/>
+      <c r="Q102" s="10" t="n"/>
+      <c r="R102" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Pucallpa – Ucayali living landscape (PER-PCL), used to define the landscape across the catalogue. Source: INEI referential census district limits (cartography of the V Censo Nacional Economico 2022; 'Distrital' layer, ide.inei.gob.pe): 11 whole districts of Coronel Portillo and Padre Abad provinces (Ucayali) and a clipped part of Calleria. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S102" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T102" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U102" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V102" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/PER-PCL_Pucallpa_Ucayali_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W102" s="10" t="inlineStr">
+        <is>
+          <t>82 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-104</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>Fatick Department living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>SEN-FK — Fatick Department</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J103" s="8" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K103" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L103" s="8" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M103" s="8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N103" s="8" t="inlineStr">
+        <is>
+          <t>SEN-FK_Fatick_Department_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O103" s="8" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P103" s="8" t="n"/>
+      <c r="Q103" s="8" t="n"/>
+      <c r="R103" s="9" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Fatick Department living landscape (SEN-FK), used to define the landscape across the catalogue. Source: GADM: level 2 unit Fatick departement (GADM v2 attribute schema; geometry identical to GADM 3.6 and 4.1 SEN.3.1_1). Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S103" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T103" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U103" s="8" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V103" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/SEN-FK_Fatick_Department_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W103" s="8" t="inlineStr">
+        <is>
+          <t>16 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-105</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Mbire – Lower Zambezi Valley living landscape boundary</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Boundaries / admin units</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>ZWE-MB — Mbire – Lower Zambezi Valley</t>
+        </is>
+      </c>
+      <c r="F104" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G104" s="10" t="inlineStr">
+        <is>
+          <t>Landscape boundary</t>
+        </is>
+      </c>
+      <c r="H104" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I104" s="10" t="inlineStr">
+        <is>
+          <t>Alliance Bioversity-CIAT (MOSAIC)</t>
+        </is>
+      </c>
+      <c r="J104" s="10" t="inlineStr">
+        <is>
+          <t>Lizeth Llanos (l.llanos@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K104" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L104" s="10" t="inlineStr">
+        <is>
+          <t>Source terms (https://gadm.org/license.html)</t>
+        </is>
+      </c>
+      <c r="M104" s="10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+      <c r="N104" s="10" t="inlineStr">
+        <is>
+          <t>ZWE-MB_Mbire_Lower_Zambezi_Valley_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="O104" s="10" t="inlineStr">
+        <is>
+          <t>GitHub release boundaries-2026-10-14 (MOSAIC-mfl/catalog)</t>
+        </is>
+      </c>
+      <c r="P104" s="10" t="n"/>
+      <c r="Q104" s="10" t="n"/>
+      <c r="R104" s="11" t="inlineStr">
+        <is>
+          <t>Canonical MOSAIC delineation of the Mbire – Lower Zambezi Valley living landscape (ZWE-MB), used to define the landscape across the catalogue. Source: GADM 4.1, level 3: all 112 wards of the districts Mbire, Centenary/Muzarabani and Mount Darwin (Mashonaland Central) and Hurungwe (Mashonaland West), unmodified. Full-detail Shapefile and GeoPackage in the dated release boundaries-2026-10-14 of MOSAIC-mfl/catalog; a simplified outline is attached to the landscape's STAC collection.</t>
+        </is>
+      </c>
+      <c r="S104" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="T104" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="U104" s="10" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="V104" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MOSAIC-mfl/catalog/releases/download/boundaries-2026-10-14/ZWE-MB_Mbire_Lower_Zambezi_Valley_boundary_2026-10-14.zip</t>
+        </is>
+      </c>
+      <c r="W104" s="10" t="inlineStr">
+        <is>
+          <t>185 KB</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:W96"/>
+  <autoFilter ref="A2:W104"/>
   <conditionalFormatting sqref="K3:K300">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Open"</formula>

</xml_diff>

<commit_message>
Set 25 records that need permission to Restricted or Internal (access level rule)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -1537,7 +1537,7 @@
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="L3" s="8" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="K22" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L22" s="10" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L24" s="10" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L25" s="8" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L27" s="8" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L29" s="8" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L30" s="10" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L32" s="10" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="K34" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L34" s="10" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="K35" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L35" s="8" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="K36" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L36" s="10" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L38" s="10" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="K40" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L40" s="10" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="K41" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L41" s="8" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="K42" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L42" s="10" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L43" s="8" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L44" s="10" t="inlineStr">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="K62" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L62" s="10" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="K64" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L64" s="10" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="K67" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L68" s="10" t="inlineStr">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L82" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Pipeline test suite and access level rule (#4)
- stdlib unittest suite (26 tests, incl. a golden rebuild test and a guard against the silent Excel fallback)
- CI pins openpyxl==3.1.5 and pyyaml==6.0.3 and runs the tests before the build in both workflows
- mosaic_pipeline/rules.py: an Open record needs a usable download_url and a licence that does not say "contact data owner"; the build aborts (exit 3) otherwise
- 25 records corrected (000, 002 -> Internal; 23 -> Restricted); see docs/RECORDS_CHANGELOG_2026-10-22_access.md
- Rollback: revert this commit; it restores the previous stac/ and datasets.json and removes the rule together

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -1537,7 +1537,7 @@
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="L3" s="8" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="K22" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L22" s="10" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L24" s="10" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L25" s="8" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L27" s="8" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L29" s="8" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L30" s="10" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L32" s="10" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="K34" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L34" s="10" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="K35" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L35" s="8" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="K36" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L36" s="10" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L38" s="10" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="K40" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L40" s="10" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="K41" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L41" s="8" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="K42" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L42" s="10" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L43" s="8" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L44" s="10" t="inlineStr">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="K62" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L62" s="10" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="K64" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L64" s="10" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="K67" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L68" s="10" t="inlineStr">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="L82" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate the Excel working view after the 039 and 041 fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -5064,7 +5064,7 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>District level crop area, prodcution and yield data - India</t>
+          <t>District level crop area, production and yield data - Ethiopia</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -5296,11 +5296,7 @@
       </c>
       <c r="P43" s="8" t="n"/>
       <c r="Q43" s="8" t="n"/>
-      <c r="R43" s="9" t="inlineStr">
-        <is>
-          <t>Agroecological zonations</t>
-        </is>
-      </c>
+      <c r="R43" s="9" t="n"/>
       <c r="S43" s="8" t="n"/>
       <c r="T43" s="8" t="n"/>
       <c r="U43" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Fix the title of 039 and the description of 041 (Omo-Gibe) (#5)
* Fix the title of 039 and the description of 041 (Omo-Gibe)

039 is Ethiopian crop data whose title was carried over from the India
record 008. 041 had the description of 040 copied into it; cleared rather
than guessed. Outputs rebuilt; tests pass. See docs/RECORDS_CHANGELOG_2026-10-28.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* Regenerate the Excel working view after the 039 and 041 fixes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

---------

Co-authored-by: lizciat <l.llanos@cgiar.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -5064,7 +5064,7 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>District level crop area, prodcution and yield data - India</t>
+          <t>District level crop area, production and yield data - Ethiopia</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -5296,11 +5296,7 @@
       </c>
       <c r="P43" s="8" t="n"/>
       <c r="Q43" s="8" t="n"/>
-      <c r="R43" s="9" t="inlineStr">
-        <is>
-          <t>Agroecological zonations</t>
-        </is>
-      </c>
+      <c r="R43" s="9" t="n"/>
       <c r="S43" s="8" t="n"/>
       <c r="T43" s="8" t="n"/>
       <c r="U43" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Point IND-CH records 013-015 to the CoRE Stack layer sheet
Their download links were QGIS style files. The CoRE Stack GEE Layers
Links sheet gives each layer's Earth Engine asset, Drive download and
licence. 014's layers are India-WRIS data re-published by CoRE Stack, so
its licence is no longer CC BY 4.0. Details in
docs/RECORDS_CHANGELOG_2026-10-29.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -2794,7 +2794,7 @@
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>National government (external)</t>
+          <t>CoRE Stack (external)</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
@@ -2821,7 +2821,7 @@
       <c r="N16" s="10" t="n"/>
       <c r="O16" s="10" t="inlineStr">
         <is>
-          <t>CoreStack: Github / Google rive</t>
+          <t>CoRE Stack: public Google Earth Engine assets and Google Drive downloads, one row per layer in the CoRE Stack GEE Layers Links sheet. Map viewer: https://ee-corestackdev.projects.earthengine.app/view/core-stack-gee-app</t>
         </is>
       </c>
       <c r="P16" s="10" t="n"/>
@@ -2844,8 +2844,7 @@
       </c>
       <c r="V16" s="10" t="inlineStr">
         <is>
-          <t>https://github.com/core-stack-org/QGIS-Styles/blob/main/Tree%20Health/ccd_style.qml
-https://github.com/core-stack-org/QGIS-Styles/blob/main/Tree%20Health/canopy_height.qml</t>
+          <t>https://docs.google.com/spreadsheets/d/1xS5d7vgyjyoqqnmmajKDZBx9qS6GqyAdSbNDR62ot2Y/edit?gid=0</t>
         </is>
       </c>
       <c r="W16" s="10" t="n"/>
@@ -2893,7 +2892,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>National government (external)</t>
+          <t>India-WRIS, via CoRE Stack (external)</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -2909,7 +2908,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>India-WRIS layers re-published by CoRE Stack; no licence stated by the source</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -2920,7 +2919,7 @@
       <c r="N17" s="8" t="n"/>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>CoreStack: Github / Google rive</t>
+          <t>CoRE Stack: public Google Earth Engine assets and Google Drive downloads, one row per layer in the CoRE Stack GEE Layers Links sheet (Waterbodies Layers group). Map viewer: https://ee-corestackdev.projects.earthengine.app/view/core-stack-gee-app</t>
         </is>
       </c>
       <c r="P17" s="8" t="n"/>
@@ -2943,7 +2942,7 @@
       </c>
       <c r="V17" s="8" t="inlineStr">
         <is>
-          <t>https://github.com/core-stack-org/QGIS-Styles/blob/main/Hydrology/Sub-Basin_style.qml</t>
+          <t>https://docs.google.com/spreadsheets/d/1xS5d7vgyjyoqqnmmajKDZBx9qS6GqyAdSbNDR62ot2Y/edit?gid=0</t>
         </is>
       </c>
       <c r="W17" s="8" t="n"/>
@@ -2991,7 +2990,7 @@
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>National government (external)</t>
+          <t>CoRE Stack (external)</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
@@ -3018,7 +3017,7 @@
       <c r="N18" s="10" t="n"/>
       <c r="O18" s="10" t="inlineStr">
         <is>
-          <t>CoreStack: Github / Google rive</t>
+          <t>CoRE Stack: public Google Earth Engine assets and Google Drive downloads, one row per layer in the CoRE Stack GEE Layers Links sheet. Map viewer: https://ee-corestackdev.projects.earthengine.app/view/core-stack-gee-app</t>
         </is>
       </c>
       <c r="P18" s="10" t="n"/>
@@ -3041,7 +3040,7 @@
       </c>
       <c r="V18" s="10" t="inlineStr">
         <is>
-          <t>https://github.com/core-stack-org/QGIS-Styles/blob/main/Land/LULC0_12class.qml</t>
+          <t>https://docs.google.com/spreadsheets/d/1xS5d7vgyjyoqqnmmajKDZBx9qS6GqyAdSbNDR62ot2Y/edit?gid=0</t>
         </is>
       </c>
       <c r="W18" s="10" t="n"/>

</xml_diff>

<commit_message>
Point IND-CH records 013-015 to the CoRE Stack layer sheet (#6)
Their download links were QGIS style files. The CoRE Stack GEE Layers
Links sheet gives each layer's Earth Engine asset, Drive download and
licence. 014's layers are India-WRIS data re-published by CoRE Stack, so
its licence is no longer CC BY 4.0. Details in
docs/RECORDS_CHANGELOG_2026-10-29.md.

Co-authored-by: lizciat <l.llanos@cgiar.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -2794,7 +2794,7 @@
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>National government (external)</t>
+          <t>CoRE Stack (external)</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
@@ -2821,7 +2821,7 @@
       <c r="N16" s="10" t="n"/>
       <c r="O16" s="10" t="inlineStr">
         <is>
-          <t>CoreStack: Github / Google rive</t>
+          <t>CoRE Stack: public Google Earth Engine assets and Google Drive downloads, one row per layer in the CoRE Stack GEE Layers Links sheet. Map viewer: https://ee-corestackdev.projects.earthengine.app/view/core-stack-gee-app</t>
         </is>
       </c>
       <c r="P16" s="10" t="n"/>
@@ -2844,8 +2844,7 @@
       </c>
       <c r="V16" s="10" t="inlineStr">
         <is>
-          <t>https://github.com/core-stack-org/QGIS-Styles/blob/main/Tree%20Health/ccd_style.qml
-https://github.com/core-stack-org/QGIS-Styles/blob/main/Tree%20Health/canopy_height.qml</t>
+          <t>https://docs.google.com/spreadsheets/d/1xS5d7vgyjyoqqnmmajKDZBx9qS6GqyAdSbNDR62ot2Y/edit?gid=0</t>
         </is>
       </c>
       <c r="W16" s="10" t="n"/>
@@ -2893,7 +2892,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>National government (external)</t>
+          <t>India-WRIS, via CoRE Stack (external)</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -2909,7 +2908,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>India-WRIS layers re-published by CoRE Stack; no licence stated by the source</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -2920,7 +2919,7 @@
       <c r="N17" s="8" t="n"/>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>CoreStack: Github / Google rive</t>
+          <t>CoRE Stack: public Google Earth Engine assets and Google Drive downloads, one row per layer in the CoRE Stack GEE Layers Links sheet (Waterbodies Layers group). Map viewer: https://ee-corestackdev.projects.earthengine.app/view/core-stack-gee-app</t>
         </is>
       </c>
       <c r="P17" s="8" t="n"/>
@@ -2943,7 +2942,7 @@
       </c>
       <c r="V17" s="8" t="inlineStr">
         <is>
-          <t>https://github.com/core-stack-org/QGIS-Styles/blob/main/Hydrology/Sub-Basin_style.qml</t>
+          <t>https://docs.google.com/spreadsheets/d/1xS5d7vgyjyoqqnmmajKDZBx9qS6GqyAdSbNDR62ot2Y/edit?gid=0</t>
         </is>
       </c>
       <c r="W17" s="8" t="n"/>
@@ -2991,7 +2990,7 @@
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>National government (external)</t>
+          <t>CoRE Stack (external)</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
@@ -3018,7 +3017,7 @@
       <c r="N18" s="10" t="n"/>
       <c r="O18" s="10" t="inlineStr">
         <is>
-          <t>CoreStack: Github / Google rive</t>
+          <t>CoRE Stack: public Google Earth Engine assets and Google Drive downloads, one row per layer in the CoRE Stack GEE Layers Links sheet. Map viewer: https://ee-corestackdev.projects.earthengine.app/view/core-stack-gee-app</t>
         </is>
       </c>
       <c r="P18" s="10" t="n"/>
@@ -3041,7 +3040,7 @@
       </c>
       <c r="V18" s="10" t="inlineStr">
         <is>
-          <t>https://github.com/core-stack-org/QGIS-Styles/blob/main/Land/LULC0_12class.qml</t>
+          <t>https://docs.google.com/spreadsheets/d/1xS5d7vgyjyoqqnmmajKDZBx9qS6GqyAdSbNDR62ot2Y/edit?gid=0</t>
         </is>
       </c>
       <c r="W18" s="10" t="n"/>

</xml_diff>